<commit_message>
fix(eval-008): the sheet accepts the rubric's whole 1-5 scale
The dropdown offered 1/3/5, the three points carrying worded anchors.
The rubric says "use 2 and 4 for anything in between", so the sheet
refused values the pre-registered instrument invites — and eval-006
reports quadratic-weighted kappa over the scale actually used, making
this a silent change to the analysis rather than a stricter sheet.

The test asserted the assumption, not the rubric, and was green.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/measurements/corpus/scoring_pack/score_sheet.xlsx
+++ b/backend/measurements/corpus/scoring_pack/score_sheet.xlsx
@@ -159,7 +159,8 @@
 Does it actually reason from the evidence, or just repeat it?
 1 = Repeats the findings back, or ignores them. No reasoning connects the evidence to the conclusion.
 3 = Uses the findings correctly, but in a generic way -- the same words would fit many different situations.
-5 = Reasons from these specific findings, connects them to each other, and shows how they lead to the conclusion.</t>
+5 = Reasons from these specific findings, connects them to each other, and shows how they lead to the conclusion.
+Use 2 and 4 for anything in between.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -168,7 +169,8 @@
 Is it honest about what it doesn't know?
 1 = No uncertainty stated, or a boilerplate disclaimer that would apply to any output whatsoever.
 3 = Names a real uncertainty, but doesn't say what difference it makes.
-5 = Names specific uncertainties and explains how each one weakens or qualifies the conclusion.</t>
+5 = Names specific uncertainties and explains how each one weakens or qualifies the conclusion.
+Use 2 and 4 for anything in between.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
@@ -177,7 +179,8 @@
 Does it offer genuine competing possibilities?
 1 = None offered, or the 'alternatives' are restatements of the main explanation.
 3 = Plausible alternatives listed, but nothing said about how you'd tell them apart.
-5 = Genuine competing explanations, with an indication of what evidence would distinguish them.</t>
+5 = Genuine competing explanations, with an indication of what evidence would distinguish them.
+Use 2 and 4 for anything in between.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
@@ -186,7 +189,8 @@
 Could an analyst act on this?
 1 = No action, or something so generic it carries no information ('investigate further').
 3 = Sensible, but non-specific -- right direction, no concrete step.
-5 = A specific next step, appropriate to this evidence, that an analyst could take immediately.</t>
+5 = A specific next step, appropriate to this evidence, that an analyst could take immediately.
+Use 2 and 4 for anything in between.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -195,7 +199,8 @@
 Would this help an analyst working under time pressure? Your overall judgement, not an average of the other four.
 1 = Would waste time, or point in the wrong direction.
 3 = Mildly helpful. Saves a little work.
-5 = Would meaningfully speed up correct triage.</t>
+5 = Would meaningfully speed up correct triage.
+Use 2 and 4 for anything in between.</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
@@ -1539,20 +1544,20 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <dataValidations count="7">
-    <dataValidation sqref="D2:D41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the scale" error="Choose one of: 1, 3, 5" type="list">
-      <formula1>"1,3,5"</formula1>
+    <dataValidation sqref="D2:D41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the scale" error="Choose one of: 1, 2, 3, 4, 5" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the scale" error="Choose one of: 1, 3, 5" type="list">
-      <formula1>"1,3,5"</formula1>
+    <dataValidation sqref="E2:E41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the scale" error="Choose one of: 1, 2, 3, 4, 5" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the scale" error="Choose one of: 1, 3, 5" type="list">
-      <formula1>"1,3,5"</formula1>
+    <dataValidation sqref="F2:F41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the scale" error="Choose one of: 1, 2, 3, 4, 5" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the scale" error="Choose one of: 1, 3, 5" type="list">
-      <formula1>"1,3,5"</formula1>
+    <dataValidation sqref="G2:G41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the scale" error="Choose one of: 1, 2, 3, 4, 5" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the scale" error="Choose one of: 1, 3, 5" type="list">
-      <formula1>"1,3,5"</formula1>
+    <dataValidation sqref="H2:H41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the scale" error="Choose one of: 1, 2, 3, 4, 5" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I41" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Not on the scale" error="Choose one of: Correct, Partly correct, Incorrect" type="list">
       <formula1>"Correct,Partly correct,Incorrect"</formula1>
@@ -1572,7 +1577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1644,256 +1649,272 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2 and 4</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Anything in between the worded points.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Uncertainty</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Is it honest about what it doesn't know?</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>No uncertainty stated, or a boilerplate disclaimer that would apply to any output whatsoever.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Names a real uncertainty, but doesn't say what difference it makes.</t>
+          <t>No uncertainty stated, or a boilerplate disclaimer that would apply to any output whatsoever.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Names a real uncertainty, but doesn't say what difference it makes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Names specific uncertainties and explains how each one weakens or qualifies the conclusion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Alternative explanations</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Does it offer genuine competing possibilities?</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
-      <c r="B11" t="n">
-        <v>1</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2 and 4</t>
+        </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>None offered, or the 'alternatives' are restatements of the main explanation.</t>
+          <t>Anything in between the worded points.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="n">
-        <v>3</v>
-      </c>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Alternative explanations</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Plausible alternatives listed, but nothing said about how you'd tell them apart.</t>
+          <t>Does it offer genuine competing possibilities?</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Genuine competing explanations, with an indication of what evidence would distinguish them.</t>
+          <t>None offered, or the 'alternatives' are restatements of the main explanation.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Recommended action</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Could an analyst act on this?</t>
+          <t>Plausible alternatives listed, but nothing said about how you'd tell them apart.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>No action, or something so generic it carries no information ('investigate further').</t>
+          <t>Genuine competing explanations, with an indication of what evidence would distinguish them.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
-      <c r="B16" t="n">
-        <v>3</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2 and 4</t>
+        </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Sensible, but non-specific -- right direction, no concrete step.</t>
+          <t>Anything in between the worded points.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="n">
-        <v>5</v>
-      </c>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Recommended action</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>A specific next step, appropriate to this evidence, that an analyst could take immediately.</t>
+          <t>Could an analyst act on this?</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Overall usefulness</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Would this help an analyst working under time pressure? Your overall judgement, not an average of the other four.</t>
+          <t>No action, or something so generic it carries no information ('investigate further').</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Would waste time, or point in the wrong direction.</t>
+          <t>Sensible, but non-specific -- right direction, no concrete step.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Mildly helpful. Saves a little work.</t>
+          <t>A specific next step, appropriate to this evidence, that an analyst could take immediately.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
-      <c r="B21" t="n">
-        <v>5</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2 and 4</t>
+        </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Would meaningfully speed up correct triage.</t>
+          <t>Anything in between the worded points.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Cause correctness</t>
+          <t>Overall usefulness</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>SECOND PASS ONLY. Does the explanation identify what was actually happening?</t>
+          <t>Would this help an analyst working under time pressure? Your overall judgement, not an average of the other four.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Correct</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr"/>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Would waste time, or point in the wrong direction.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Partly correct</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr"/>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Mildly helpful. Saves a little work.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Incorrect</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr"/>
+      <c r="B25" t="n">
+        <v>5</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Would meaningfully speed up correct triage.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Confidence calibration</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2 and 4</t>
+        </is>
+      </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>SECOND PASS ONLY. Given how strong the evidence actually was, is the stated confidence right? A confident-sounding hypothesis built on weak evidence is Too high even if it turned out correct.</t>
+          <t>Anything in between the worded points.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Too low</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr"/>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Cause correctness</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>SECOND PASS ONLY. Does the explanation identify what was actually happening?</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>About right</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr"/>
@@ -1902,10 +1923,59 @@
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
+          <t>Partly correct</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Incorrect</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Confidence calibration</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>SECOND PASS ONLY. Given how strong the evidence actually was, is the stated confidence right? A confident-sounding hypothesis built on weak evidence is Too high even if it turned out correct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Too low</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>About right</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>Too high</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(eval-009): a glossary the scorer can read mid-flow - tests pass
22 terms at the head of hypotheses.md and on a Terms sheet in the
workbook, so it is reachable both where the evidence is read and where
the score is entered.

Definitions say what a term denotes, never what it implies: a gloss
like "aircraft stopped reporting, which indicates interference" hands
over the causal link dimension 1 and pass-two cause correctness both
exist to test. Enforced by CAUSAL_CONNECTIVES, asserted over every
entry, and fired at a real violation.

A citation key with no entry is refused rather than omitted. That guard
immediately found a real drift: the bundle fixtures used
"track_discontinuity", a finding type the detection layer never emits —
renamed to track_continuity_gap across three suites.

1301 passed, app/evaluation at 100%.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/measurements/corpus/scoring_pack/score_sheet.xlsx
+++ b/backend/measurements/corpus/scoring_pack/score_sheet.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Scores" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="How to score" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Terms" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1980,4 +1981,298 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>What it refers to</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RF-NOISE</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>The rule that compares each radio reading against what that receiver normally reads on that channel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TRACK-GAP</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>The rule that looks for aircraft whose position reports stop arriving.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SENSOR-FAULT</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>The rule that compares one receiver against the receivers near it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FUSION-SPATIAL</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>The rule that reports when more than one receiver deviated in the same area and the same window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>possible_interference_zone</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>The conclusion that more than one receiver deviated at the same time in the same area.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>possible_sensor_fault</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>The conclusion that one receiver deviated while the neighbours that could be measured stayed within their normal range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>rf_noise_deviation</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>One run of consecutive readings on one receiver and one channel that sat far enough from that cell's normal to be recorded as an event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>track_continuity_gap</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>One aircraft's position reports stopping for longer than the gap the rule allows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>track_rate_excess</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>How often aircraft dropped out inside the window, set against how often they dropped out in the same area outside it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>neighbour_nominal</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>A receiver near the one under examination that was measured and stayed within its normal range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>channel_adjacency</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>How many of a receiver's channels the deviation covered, out of the total it watches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>The average and spread of what one receiver reads on one channel, worked out from quiet periods only. Every receiver and channel has its own; they are never pooled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>channel</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>One slice of the radio spectrum. Each receiver watches several, numbered from 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>dB</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Decibel, the unit these readings use. It is a ratio on a logarithmic scale: 3 dB is about double, 10 dB is ten times, 20 dB is a hundred times.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>power_dbm</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Received signal power, in decibels relative to one milliwatt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>nominal</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Within the normal range for that receiver and channel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>disc</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>A circular area of the stated radius, centred on the event, used to decide which aircraft count as near it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>discontinuity</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>One break in one aircraft's stream of position reports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>reference period</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>The time outside the event window, used as the comparison for a rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>rate ratio</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>The rate inside the window divided by the rate in the reference period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>smoothing constant</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>A small fixed number added to both sides of a rate comparison so that a division by zero cannot occur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>corroborate</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>To look for agreement from the other half of the picture -- the aircraft side for a radio finding, and the reverse. Recorded as one of three values: corroborated, measured and not corroborated, or not measurable.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>